<commit_message>
wip(catalog): customer-supplied SKUs, PO main-supplier pick, no PO for CUSTOMER lines
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/catalog-import/hookka-300t-review.xlsx
+++ b/docs/catalog-import/hookka-300t-review.xlsx
@@ -14,7 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mattresses" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Surcharges" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes vs current system" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer items" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Bedframes'!$A$1:$J$162</definedName>
@@ -498,7 +499,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sheets: Bedframes, Sofas (matrix), Mattresses, Surcharges, Changes vs current system, Questions.</t>
+          <t>Sheets: Bedframes, Sofas (matrix), Accessories, Mattresses, Surcharges, Changes vs current system, Customer items, Questions.</t>
         </is>
       </c>
     </row>
@@ -47772,7 +47773,2527 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:H65"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SKU code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Sub-category</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Cost (RM)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Purchase order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CUS-PROTECTION</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Customer Protection</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Protection</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CUS-HACKING</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Customer Hacking</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Hacking</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CUS-PLUMBING</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Customer Plumbing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CUS-WATERPROOFING</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Customer Waterproofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Waterproofing</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CUS-ELECTRICAL</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Customer Electrical</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CUS-MASONRY_TILING</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Customer Masonry / tiling</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Masonry / tiling</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CUS-PLASTER_CEILING</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Customer Plaster ceiling</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Plaster ceiling</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CUS-PARTITION</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Customer Partition</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Partition</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CUS-ALUMINIUM_GLASS</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Customer Window / sliding door / glass</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Window / sliding door / glass</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CUS-DOOR</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Customer Door</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Door</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CUS-GRILL</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Customer Grill</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Grill</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CUS-PAINTING</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Customer Painting</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Painting</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CUS-TEXTURED_PAINTING</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Customer Textured painting</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Textured painting</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CUS-FEATURE_WALL</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Customer Feature wall</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Feature wall</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CUS-FLOORING</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Customer Flooring</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Flooring</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CUS-KITCHEN_CABINET</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Customer Kitchen cabinet</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Built-in</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Kitchen cabinet</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CUS-WARDROBE</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Customer Wardrobe</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Built-in</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Wardrobe</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>CUS-TV_CABINET</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Customer TV cabinet</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Built-in</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>TV cabinet</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CUS-SHOE_CABINET</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Customer Shoe cabinet</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Built-in</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Shoe cabinet</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CUS-STUDY_TABLE</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Customer Study table</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Built-in</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Study table</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CUS-COUNTERTOP</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Customer Countertop (stone)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Built-in</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Countertop (stone)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CUS-SHELVING</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Customer Shelving</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Built-in</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Shelving</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CUS-SOFA</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Customer Sofa</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Sofa</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CUS-BEDFRAME</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Customer Bedframe</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Bedframe</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CUS-MATTRESS</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Customer Mattress</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Mattress</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CUS-DINING</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Customer Dining</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Dining</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CUS-TABLES</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Customer Tables</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Tables</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CUS-LOOSE_STORAGE</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Customer Loose storage</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Loose storage</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>CUS-ACCESSORY</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Customer Accessory</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Accessory</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CUS-DOWNLIGHT</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Customer Downlight</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Lighting</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Downlight</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>CUS-EYEBALL</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Customer Eye ball</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Lighting</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Eye ball</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>CUS-PENDANT</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Customer Pendant</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Lighting</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Pendant</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>CUS-LED_STRIP</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Customer LED strip</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Lighting</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>LED strip</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>CUS-CEILING_FAN</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Customer Ceiling fan</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Lighting</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Ceiling fan</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>CUS-TRACK_LIGHT</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Customer Track light</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Lighting</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Track light</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>CUS-TV</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Customer TV</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Appliances</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>TV</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>CUS-FRIDGE</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Customer Fridge</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Appliances</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Fridge</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>CUS-WASHER</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Customer Washer</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Appliances</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Washer</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>CUS-WATER_HEATER</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Customer Water heater</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Appliances</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Water heater</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>CUS-HOOD_HOB</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Customer Hood / hob</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Appliances</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Hood / hob</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>CUS-AIRCON_UNIT</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Customer Aircon unit</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Appliances</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Aircon unit</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>CUS-CURTAIN_BLINDS</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Customer Curtain / blinds</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Soft furnishing</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Curtain / blinds</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CUS-BED_LINEN</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Customer Bed linen</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Soft furnishing</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Bed linen</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>CUS-AMENITIES</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Customer Amenities</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Soft furnishing</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Amenities</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>CUS-DECORATION</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Customer Decoration</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Soft furnishing</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Decoration</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>CUS-CARPET</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Customer Carpet</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Soft furnishing</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Carpet</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>CUS-DIFFUSER</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Customer Diffuser</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Soft furnishing</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Diffuser</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>CUS-DELIVERY</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Customer Delivery</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>CUS-STYLING</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Customer Styling</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Styling</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>CUS-PHOTOSHOOT</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Customer Photoshoot</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Photoshoot</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>CUS-AIRBNB_SETUP</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Customer Airbnb setup</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Airbnb setup</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>CUS-AIRCON_INSTALL</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Customer Aircon install</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Aircon install</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>CUS-CLEANING</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Customer Cleaning</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Cleaning</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>CUS-PROJECT_MGMT</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Customer Project management</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Project management</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>CUS-WORKS</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Customer Works</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Works</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Protection (group item)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>CUS-BUILTIN</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Customer Built-in</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Built-in</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Shelving (group item)</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>CUS-FURNITURE</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Customer Furniture</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Loose storage (group item)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>CUS-LIGHTING</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Customer Lighting</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Lighting</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Downlight (group item)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>CUS-APPLIANCE</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Customer Appliance</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Appliances</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>TV (group item)</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>CUS-SOFT</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Customer Soft furnishing</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Soft furnishing</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Decoration (group item)</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>CUS-SERVICE</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Customer Service</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>(group item)</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>UNIT</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>never raised from a renovation contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>54 sub-categories on a database built from the migrations (production has 55 after 0141): the migration reads the sub-categories when it runs, so every active one on production gets its Customer SKU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Meaning: the customer orders / handles this item; The Conts manages it on the project. Supplier CUSTOMER, cost RM 0.00 on purpose (not "price needed"). A renovation contract line with a Customer SKU is skipped when purchase orders are raised.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -47968,12 +50489,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>HOOKKA lists sofa seat sizes 44, 24" x 37" and 12 that no quoted price uses.</t>
+          <t>Customer items per group sit under one sub-category each (Works &gt; Protection, Built-in &gt; Shelving, Furniture &gt; Loose storage, Lighting &gt; Downlight, Appliances &gt; TV, Soft furnishing &gt; Decoration; Service needs none). The engine needs a sub-category for every group but Service. Better homes for them?</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Not added to the sizes list.</t>
+          <t>As listed on the Customer items sheet.</t>
         </is>
       </c>
     </row>
@@ -47983,12 +50504,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Surcharges that differ from Products &gt; Maintenance (copied from Houzs): see the Surcharges sheet. Should the master take HOOKKA's values?</t>
+          <t>HOOKKA lists sofa seat sizes 44, 24" x 37" and 12 that no quoted price uses.</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>HOOKKA purchase orders use HOOKKA's values; sales-order costing keeps the master values.</t>
+          <t>Not added to the sizes list.</t>
         </is>
       </c>
     </row>
@@ -47998,12 +50519,12 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>41 HOOKKA SKUs of the old catalogue are not on the quotation (e.g. 1003-(SK) and 1003-(220X220): the quotation has those sizes only under 1003(A); the 1009 family is now 1009(A); DIVAN sizes are coded by HOOKKA as DIVAN-(153) etc.).</t>
+          <t>Surcharges that differ from Products &gt; Maintenance (copied from Houzs): see the Surcharges sheet. Should the master take HOOKKA's values?</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Removed (see Changes).</t>
+          <t>HOOKKA purchase orders use HOOKKA's values; sales-order costing keeps the master values.</t>
         </is>
       </c>
     </row>
@@ -48013,10 +50534,25 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
+          <t>41 HOOKKA SKUs of the old catalogue are not on the quotation (e.g. 1003-(SK) and 1003-(220X220): the quotation has those sizes only under 1003(A); the 1009 family is now 1009(A); DIVAN sizes are coded by HOOKKA as DIVAN-(153) etc.).</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Removed (see Changes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
           <t>AKEMI: 39 rows have no price: every CUSTOM (SP) size, plus HS SOLACE 200x200 and all 5 KORI IYASHI sizes.</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Created and linked to Houzs Century with cost 0, "PRICE NEEDED".</t>
         </is>

</xml_diff>